<commit_message>
Agregando modificaciones de rutaactual e inventario
Agregando funcionalidad de visualizacion de inventarios de insumos en furgon tanto en inventarios como en ruta actual. funcionalidades propias agregadas (sumar, descontar insumo, confirmar, a ruta, etc)
</commit_message>
<xml_diff>
--- a/bd/mediclean_bd.xlsx
+++ b/bd/mediclean_bd.xlsx
@@ -618,7 +618,7 @@
       </c>
       <c r="C2" s="18" t="inlineStr">
         <is>
-          <t>tFPY7eL_FZCzga9igM2pUz_cZiUBH_UWsX7BjmyzKCw</t>
+          <t>OPwt2ePEWlCHNbtcSEe4ysnHeYxLyBaMpMPC4hozSq8</t>
         </is>
       </c>
     </row>
@@ -1153,7 +1153,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K191"/>
+  <dimension ref="A1:K187"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.5859375" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="15" min="1" max="1"/>
@@ -9788,186 +9788,6 @@
       <c r="I187" s="15" t="inlineStr">
         <is>
           <t>contacto, sra Marcia Carmona</t>
-        </is>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" s="15" t="n">
-        <v>10185</v>
-      </c>
-      <c r="B188" s="15" t="inlineStr">
-        <is>
-          <t>activo</t>
-        </is>
-      </c>
-      <c r="C188" s="15" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="D188" s="15" t="inlineStr">
-        <is>
-          <t>77.884.397-8</t>
-        </is>
-      </c>
-      <c r="E188" s="15" t="inlineStr">
-        <is>
-          <t>centro odontologico carvajal y fernandez ltda</t>
-        </is>
-      </c>
-      <c r="F188" s="15" t="inlineStr">
-        <is>
-          <t>o´higgins 485 of 408</t>
-        </is>
-      </c>
-      <c r="G188" s="15" t="inlineStr">
-        <is>
-          <t>Osorno</t>
-        </is>
-      </c>
-      <c r="H188" s="15" t="inlineStr">
-        <is>
-          <t>975643988/971381140</t>
-        </is>
-      </c>
-      <c r="I188" s="15" t="inlineStr">
-        <is>
-          <t>cliente ingresado automaticamente</t>
-        </is>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" s="15" t="n">
-        <v>10186</v>
-      </c>
-      <c r="B189" s="15" t="inlineStr">
-        <is>
-          <t>activo</t>
-        </is>
-      </c>
-      <c r="C189" s="15" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="D189" s="15" t="inlineStr">
-        <is>
-          <t>77.016.887-2</t>
-        </is>
-      </c>
-      <c r="E189" s="15" t="inlineStr">
-        <is>
-          <t>Oro.odontologia especializada dra natalia marti</t>
-        </is>
-      </c>
-      <c r="F189" s="15" t="inlineStr">
-        <is>
-          <t>arturo prat 662</t>
-        </is>
-      </c>
-      <c r="G189" s="15" t="inlineStr">
-        <is>
-          <t>La Union</t>
-        </is>
-      </c>
-      <c r="H189" s="15" t="inlineStr">
-        <is>
-          <t>972698736</t>
-        </is>
-      </c>
-      <c r="I189" s="15" t="inlineStr">
-        <is>
-          <t>cliente ingresado automaticamente</t>
-        </is>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" s="15" t="n">
-        <v>10187</v>
-      </c>
-      <c r="B190" s="15" t="inlineStr">
-        <is>
-          <t>activo</t>
-        </is>
-      </c>
-      <c r="C190" s="15" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="D190" s="15" t="inlineStr">
-        <is>
-          <t>77.018.394-4</t>
-        </is>
-      </c>
-      <c r="E190" s="15" t="inlineStr">
-        <is>
-          <t>Servicios Medicos Limitada</t>
-        </is>
-      </c>
-      <c r="F190" s="15" t="inlineStr">
-        <is>
-          <t>Arauco561, OF 701</t>
-        </is>
-      </c>
-      <c r="G190" s="15" t="inlineStr">
-        <is>
-          <t>Valdivia</t>
-        </is>
-      </c>
-      <c r="H190" s="15" t="inlineStr">
-        <is>
-          <t>966670399</t>
-        </is>
-      </c>
-      <c r="I190" s="15" t="inlineStr">
-        <is>
-          <t>cliente ingresado automaticamente</t>
-        </is>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" s="15" t="n">
-        <v>10188</v>
-      </c>
-      <c r="B191" s="15" t="inlineStr">
-        <is>
-          <t>activo</t>
-        </is>
-      </c>
-      <c r="C191" s="15" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="D191" s="15" t="inlineStr">
-        <is>
-          <t>6.576.720-1</t>
-        </is>
-      </c>
-      <c r="E191" s="15" t="inlineStr">
-        <is>
-          <t>Maria isabel Moreno Vivanco (medodonta)</t>
-        </is>
-      </c>
-      <c r="F191" s="15" t="inlineStr">
-        <is>
-          <t>Manuel Montt 0253</t>
-        </is>
-      </c>
-      <c r="G191" s="15" t="inlineStr">
-        <is>
-          <t>Valdivia</t>
-        </is>
-      </c>
-      <c r="H191" s="15" t="inlineStr">
-        <is>
-          <t>998295798</t>
-        </is>
-      </c>
-      <c r="I191" s="15" t="inlineStr">
-        <is>
-          <t>cliente ingresado automaticamente</t>
         </is>
       </c>
     </row>
@@ -11428,7 +11248,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AN432"/>
+  <dimension ref="A1:AN409"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.5859375" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8.699999999999999" customWidth="1" style="15" min="1" max="1"/>
@@ -28738,7 +28558,7 @@
       </c>
       <c r="K238" s="15" t="inlineStr">
         <is>
-          <t>REALIZADO</t>
+          <t>enruta</t>
         </is>
       </c>
       <c r="L238" s="15" t="inlineStr">
@@ -31235,7 +31055,7 @@
       </c>
       <c r="K275" s="15" t="inlineStr">
         <is>
-          <t>REALIZADO</t>
+          <t>enruta</t>
         </is>
       </c>
       <c r="L275" s="15" t="inlineStr">
@@ -31436,7 +31256,7 @@
       </c>
       <c r="K278" s="15" t="inlineStr">
         <is>
-          <t>REALIZADO</t>
+          <t>enruta</t>
         </is>
       </c>
       <c r="L278" s="15" t="inlineStr">
@@ -31504,7 +31324,7 @@
       </c>
       <c r="K279" s="15" t="inlineStr">
         <is>
-          <t>REALIZADO</t>
+          <t>enruta</t>
         </is>
       </c>
       <c r="L279" s="15" t="inlineStr">
@@ -32146,7 +31966,7 @@
       </c>
       <c r="K288" s="15" t="inlineStr">
         <is>
-          <t>REALIZADO</t>
+          <t>enruta</t>
         </is>
       </c>
       <c r="L288" s="15" t="inlineStr">
@@ -38262,7 +38082,7 @@
       </c>
       <c r="K378" s="15" t="inlineStr">
         <is>
-          <t>REALIZADO</t>
+          <t>enruta</t>
         </is>
       </c>
       <c r="L378" s="15" t="inlineStr">
@@ -40323,1407 +40143,6 @@
       <c r="AI409" s="15" t="inlineStr">
         <is>
           <t>Ruta: VeterinariaReloncavi-RedesClinic-CambioAceite</t>
-        </is>
-      </c>
-    </row>
-    <row r="410">
-      <c r="A410" s="15" t="inlineStr">
-        <is>
-          <t>20260203</t>
-        </is>
-      </c>
-      <c r="B410" s="15" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C410" s="15" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="D410" s="15" t="inlineStr">
-        <is>
-          <t>76.091.665-k</t>
-        </is>
-      </c>
-      <c r="E410" s="15" t="inlineStr">
-        <is>
-          <t>iglesias y maldonado ltda</t>
-        </is>
-      </c>
-      <c r="F410" s="15" t="inlineStr">
-        <is>
-          <t>Barros arana 1350 of 1</t>
-        </is>
-      </c>
-      <c r="G410" s="15" t="inlineStr">
-        <is>
-          <t>Osorno</t>
-        </is>
-      </c>
-      <c r="H410" s="15" t="inlineStr">
-        <is>
-          <t>985960741</t>
-        </is>
-      </c>
-      <c r="I410" s="15" t="inlineStr">
-        <is>
-          <t>09:00 a 12:30 y de 15:00 a 19:00.</t>
-        </is>
-      </c>
-      <c r="J410" s="15" t="n">
-        <v>10017</v>
-      </c>
-      <c r="K410" s="15" t="inlineStr">
-        <is>
-          <t>REALIZADO</t>
-        </is>
-      </c>
-      <c r="L410" s="15" t="inlineStr">
-        <is>
-          <t>ca3l1 ba1</t>
-        </is>
-      </c>
-      <c r="Z410" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF410" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="AI410" s="15" t="inlineStr">
-        <is>
-          <t>Ruta: Osorno-LaUnion-RioBueno-Valdivia</t>
-        </is>
-      </c>
-    </row>
-    <row r="411">
-      <c r="A411" s="15" t="inlineStr">
-        <is>
-          <t>20260203</t>
-        </is>
-      </c>
-      <c r="B411" s="15" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C411" s="15" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="D411" s="15" t="inlineStr">
-        <is>
-          <t>78.106.156-5</t>
-        </is>
-      </c>
-      <c r="E411" s="15" t="inlineStr">
-        <is>
-          <t>sociedad odontologica dental Fresh spa</t>
-        </is>
-      </c>
-      <c r="F411" s="15" t="inlineStr">
-        <is>
-          <t>freire 624 of 312</t>
-        </is>
-      </c>
-      <c r="G411" s="15" t="inlineStr">
-        <is>
-          <t>Osorno</t>
-        </is>
-      </c>
-      <c r="H411" s="15" t="inlineStr">
-        <is>
-          <t>950105603/990056747</t>
-        </is>
-      </c>
-      <c r="I411" s="15" t="inlineStr">
-        <is>
-          <t>9 a 13 y 14 a 20</t>
-        </is>
-      </c>
-      <c r="J411" s="15" t="n">
-        <v>10016</v>
-      </c>
-      <c r="K411" s="15" t="inlineStr">
-        <is>
-          <t>enruta</t>
-        </is>
-      </c>
-      <c r="L411" s="15" t="inlineStr">
-        <is>
-          <t>ca3l10 ba10</t>
-        </is>
-      </c>
-      <c r="Z411" s="15" t="n">
-        <v>10</v>
-      </c>
-      <c r="AF411" s="15" t="n">
-        <v>10</v>
-      </c>
-      <c r="AI411" s="15" t="inlineStr">
-        <is>
-          <t>Ruta: Osorno-LaUnion-RioBueno-Valdivia</t>
-        </is>
-      </c>
-    </row>
-    <row r="412">
-      <c r="A412" s="15" t="inlineStr">
-        <is>
-          <t>20260203</t>
-        </is>
-      </c>
-      <c r="B412" s="15" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="C412" s="15" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="D412" s="15" t="inlineStr">
-        <is>
-          <t>77.141.505-9</t>
-        </is>
-      </c>
-      <c r="E412" s="15" t="inlineStr">
-        <is>
-          <t>centro odont. Familiar Ultradens</t>
-        </is>
-      </c>
-      <c r="F412" s="15" t="inlineStr">
-        <is>
-          <t>Ramirez 684</t>
-        </is>
-      </c>
-      <c r="G412" s="15" t="inlineStr">
-        <is>
-          <t>Osorno</t>
-        </is>
-      </c>
-      <c r="H412" s="15" t="inlineStr">
-        <is>
-          <t>933892771</t>
-        </is>
-      </c>
-      <c r="I412" s="15" t="inlineStr">
-        <is>
-          <t>9:30 a 13 y 15 a 19</t>
-        </is>
-      </c>
-      <c r="J412" s="15" t="n">
-        <v>10112</v>
-      </c>
-      <c r="K412" s="15" t="inlineStr">
-        <is>
-          <t>enruta</t>
-        </is>
-      </c>
-      <c r="AI412" s="15" t="inlineStr">
-        <is>
-          <t>Ruta: Osorno-LaUnion-RioBueno-Valdivia</t>
-        </is>
-      </c>
-    </row>
-    <row r="413">
-      <c r="A413" s="15" t="inlineStr">
-        <is>
-          <t>20260203</t>
-        </is>
-      </c>
-      <c r="B413" s="15" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C413" s="15" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="D413" s="15" t="inlineStr">
-        <is>
-          <t>76.828.443-1</t>
-        </is>
-      </c>
-      <c r="E413" s="15" t="inlineStr">
-        <is>
-          <t>Servicios Odontologicos CRD SpA</t>
-        </is>
-      </c>
-      <c r="F413" s="15" t="inlineStr">
-        <is>
-          <t>Pasaje Consistorial, local K</t>
-        </is>
-      </c>
-      <c r="G413" s="15" t="inlineStr">
-        <is>
-          <t>Osorno</t>
-        </is>
-      </c>
-      <c r="H413" s="15" t="inlineStr">
-        <is>
-          <t>998422751</t>
-        </is>
-      </c>
-      <c r="I413" s="15" t="inlineStr">
-        <is>
-          <t>10 A 14 Y 15 A 20</t>
-        </is>
-      </c>
-      <c r="J413" s="15" t="n">
-        <v>10014</v>
-      </c>
-      <c r="K413" s="15" t="inlineStr">
-        <is>
-          <t>enruta</t>
-        </is>
-      </c>
-      <c r="AI413" s="15" t="inlineStr">
-        <is>
-          <t>Ruta: Osorno-LaUnion-RioBueno-Valdivia</t>
-        </is>
-      </c>
-    </row>
-    <row r="414">
-      <c r="A414" s="15" t="inlineStr">
-        <is>
-          <t>20260203</t>
-        </is>
-      </c>
-      <c r="B414" s="15" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="C414" s="15" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="D414" s="15" t="inlineStr">
-        <is>
-          <t>76.958.988-0</t>
-        </is>
-      </c>
-      <c r="E414" s="15" t="inlineStr">
-        <is>
-          <t>clinica veterinaria Mundo animal</t>
-        </is>
-      </c>
-      <c r="F414" s="15" t="inlineStr">
-        <is>
-          <t>Zenteno 2748</t>
-        </is>
-      </c>
-      <c r="G414" s="15" t="inlineStr">
-        <is>
-          <t>Osorno</t>
-        </is>
-      </c>
-      <c r="H414" s="15" t="inlineStr">
-        <is>
-          <t>6442264990/990004454</t>
-        </is>
-      </c>
-      <c r="I414" s="15" t="inlineStr">
-        <is>
-          <t>10 a 14 y 15 a 19/ monserrat</t>
-        </is>
-      </c>
-      <c r="J414" s="15" t="n">
-        <v>10015</v>
-      </c>
-      <c r="K414" s="15" t="inlineStr">
-        <is>
-          <t>enruta</t>
-        </is>
-      </c>
-      <c r="AI414" s="15" t="inlineStr">
-        <is>
-          <t>Ruta: Osorno-LaUnion-RioBueno-Valdivia</t>
-        </is>
-      </c>
-    </row>
-    <row r="415">
-      <c r="A415" s="15" t="inlineStr">
-        <is>
-          <t>20260203</t>
-        </is>
-      </c>
-      <c r="B415" s="15" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="C415" s="15" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="D415" s="15" t="inlineStr">
-        <is>
-          <t>76.792.132-2</t>
-        </is>
-      </c>
-      <c r="E415" s="15" t="inlineStr">
-        <is>
-          <t>Giacomozzi y Paves ltda</t>
-        </is>
-      </c>
-      <c r="F415" s="15" t="inlineStr">
-        <is>
-          <t>Gillermo buhler 1561</t>
-        </is>
-      </c>
-      <c r="G415" s="15" t="inlineStr">
-        <is>
-          <t>Osorno</t>
-        </is>
-      </c>
-      <c r="H415" s="15" t="inlineStr">
-        <is>
-          <t>977491966/952115168</t>
-        </is>
-      </c>
-      <c r="I415" s="15" t="inlineStr">
-        <is>
-          <t>ultimo retiro febrero 2025</t>
-        </is>
-      </c>
-      <c r="J415" s="15" t="n">
-        <v>10035</v>
-      </c>
-      <c r="K415" s="15" t="inlineStr">
-        <is>
-          <t>enruta</t>
-        </is>
-      </c>
-      <c r="AI415" s="15" t="inlineStr">
-        <is>
-          <t>Ruta: Osorno-LaUnion-RioBueno-Valdivia</t>
-        </is>
-      </c>
-    </row>
-    <row r="416">
-      <c r="A416" s="15" t="inlineStr">
-        <is>
-          <t>20260203</t>
-        </is>
-      </c>
-      <c r="B416" s="15" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="C416" s="15" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="D416" s="15" t="inlineStr">
-        <is>
-          <t>65.104.083-3</t>
-        </is>
-      </c>
-      <c r="E416" s="15" t="inlineStr">
-        <is>
-          <t>Fundacion Proseger, Servicio Geriatrico</t>
-        </is>
-      </c>
-      <c r="F416" s="15" t="inlineStr">
-        <is>
-          <t>Mackenna 1040</t>
-        </is>
-      </c>
-      <c r="G416" s="15" t="inlineStr">
-        <is>
-          <t>Osorno</t>
-        </is>
-      </c>
-      <c r="H416" s="15" t="inlineStr">
-        <is>
-          <t>642481595</t>
-        </is>
-      </c>
-      <c r="I416" s="15" t="inlineStr">
-        <is>
-          <t>con deuda o problema</t>
-        </is>
-      </c>
-      <c r="J416" s="15" t="n">
-        <v>10019</v>
-      </c>
-      <c r="K416" s="15" t="inlineStr">
-        <is>
-          <t>POSPUESTO</t>
-        </is>
-      </c>
-      <c r="L416" s="15" t="inlineStr">
-        <is>
-          <t>con deuda o problema</t>
-        </is>
-      </c>
-      <c r="AI416" s="15" t="inlineStr">
-        <is>
-          <t>Ruta: Osorno-LaUnion-RioBueno-Valdivia</t>
-        </is>
-      </c>
-    </row>
-    <row r="417">
-      <c r="A417" s="15" t="inlineStr">
-        <is>
-          <t>20260203</t>
-        </is>
-      </c>
-      <c r="B417" s="15" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="C417" s="15" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="D417" s="15" t="inlineStr">
-        <is>
-          <t>77.884.397-8</t>
-        </is>
-      </c>
-      <c r="E417" s="15" t="inlineStr">
-        <is>
-          <t>centro odontologico carvajal y fernandez ltda</t>
-        </is>
-      </c>
-      <c r="F417" s="15" t="inlineStr">
-        <is>
-          <t>o´higgins 485 of 408</t>
-        </is>
-      </c>
-      <c r="G417" s="15" t="inlineStr">
-        <is>
-          <t>Osorno</t>
-        </is>
-      </c>
-      <c r="H417" s="15" t="inlineStr">
-        <is>
-          <t>975643988/971381140</t>
-        </is>
-      </c>
-      <c r="I417" s="15" t="inlineStr">
-        <is>
-          <t>con deuda o problema</t>
-        </is>
-      </c>
-      <c r="J417" s="15" t="n">
-        <v>10185</v>
-      </c>
-      <c r="K417" s="15" t="inlineStr">
-        <is>
-          <t>enruta</t>
-        </is>
-      </c>
-      <c r="AI417" s="15" t="inlineStr">
-        <is>
-          <t>Ruta: Osorno-LaUnion-RioBueno-Valdivia</t>
-        </is>
-      </c>
-    </row>
-    <row r="418">
-      <c r="A418" s="15" t="inlineStr">
-        <is>
-          <t>20260203</t>
-        </is>
-      </c>
-      <c r="B418" s="15" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="C418" s="15" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="D418" s="15" t="inlineStr">
-        <is>
-          <t>77.016.887-2</t>
-        </is>
-      </c>
-      <c r="E418" s="15" t="inlineStr">
-        <is>
-          <t>Oro.odontologia especializada dra natalia marti</t>
-        </is>
-      </c>
-      <c r="F418" s="15" t="inlineStr">
-        <is>
-          <t>arturo prat 662</t>
-        </is>
-      </c>
-      <c r="G418" s="15" t="inlineStr">
-        <is>
-          <t>La Union</t>
-        </is>
-      </c>
-      <c r="H418" s="15" t="inlineStr">
-        <is>
-          <t>972698736</t>
-        </is>
-      </c>
-      <c r="I418" s="15" t="inlineStr">
-        <is>
-          <t>10 a 13:30 y 15 a 19:30</t>
-        </is>
-      </c>
-      <c r="J418" s="15" t="n">
-        <v>10186</v>
-      </c>
-      <c r="K418" s="15" t="inlineStr">
-        <is>
-          <t>enruta</t>
-        </is>
-      </c>
-      <c r="AI418" s="15" t="inlineStr">
-        <is>
-          <t>Ruta: Osorno-LaUnion-RioBueno-Valdivia</t>
-        </is>
-      </c>
-    </row>
-    <row r="419">
-      <c r="A419" s="15" t="inlineStr">
-        <is>
-          <t>20260203</t>
-        </is>
-      </c>
-      <c r="B419" s="15" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="C419" s="15" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="D419" s="15" t="inlineStr">
-        <is>
-          <t>9999</t>
-        </is>
-      </c>
-      <c r="E419" s="15" t="inlineStr">
-        <is>
-          <t>ACHS LA UNION</t>
-        </is>
-      </c>
-      <c r="F419" s="15" t="inlineStr">
-        <is>
-          <t>Comercio Nº260, La Unión</t>
-        </is>
-      </c>
-      <c r="G419" s="15" t="inlineStr">
-        <is>
-          <t>La Union</t>
-        </is>
-      </c>
-      <c r="H419" s="15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I419" s="15" t="inlineStr">
-        <is>
-          <t>con deuda o problema: EN REMODELACION</t>
-        </is>
-      </c>
-      <c r="J419" s="15" t="n">
-        <v>10020</v>
-      </c>
-      <c r="K419" s="15" t="inlineStr">
-        <is>
-          <t>enruta</t>
-        </is>
-      </c>
-      <c r="AI419" s="15" t="inlineStr">
-        <is>
-          <t>Ruta: Osorno-LaUnion-RioBueno-Valdivia</t>
-        </is>
-      </c>
-    </row>
-    <row r="420">
-      <c r="A420" s="15" t="inlineStr">
-        <is>
-          <t>20260203</t>
-        </is>
-      </c>
-      <c r="B420" s="15" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="C420" s="15" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="D420" s="15" t="inlineStr">
-        <is>
-          <t>9999</t>
-        </is>
-      </c>
-      <c r="E420" s="15" t="inlineStr">
-        <is>
-          <t>ACHS Rio Bueno</t>
-        </is>
-      </c>
-      <c r="F420" s="15" t="inlineStr">
-        <is>
-          <t>Independencia Nº970</t>
-        </is>
-      </c>
-      <c r="G420" s="15" t="inlineStr">
-        <is>
-          <t>Rio bueno</t>
-        </is>
-      </c>
-      <c r="H420" s="15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J420" s="15" t="n">
-        <v>10021</v>
-      </c>
-      <c r="K420" s="15" t="inlineStr">
-        <is>
-          <t>enruta</t>
-        </is>
-      </c>
-      <c r="AI420" s="15" t="inlineStr">
-        <is>
-          <t>Ruta: Osorno-LaUnion-RioBueno-Valdivia</t>
-        </is>
-      </c>
-    </row>
-    <row r="421">
-      <c r="A421" s="15" t="inlineStr">
-        <is>
-          <t>20260203</t>
-        </is>
-      </c>
-      <c r="B421" s="15" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="C421" s="15" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="D421" s="15" t="inlineStr">
-        <is>
-          <t>77.574.343-3</t>
-        </is>
-      </c>
-      <c r="E421" s="15" t="inlineStr">
-        <is>
-          <t>Odontología y estética Dra Gallardo SpA</t>
-        </is>
-      </c>
-      <c r="F421" s="15" t="inlineStr">
-        <is>
-          <t>San Martín 1465</t>
-        </is>
-      </c>
-      <c r="G421" s="15" t="inlineStr">
-        <is>
-          <t>Rio bueno</t>
-        </is>
-      </c>
-      <c r="H421" s="15" t="inlineStr">
-        <is>
-          <t>940553882</t>
-        </is>
-      </c>
-      <c r="I421" s="15" t="inlineStr">
-        <is>
-          <t>10 a 14 y 15 a 19</t>
-        </is>
-      </c>
-      <c r="J421" s="15" t="n">
-        <v>10149</v>
-      </c>
-      <c r="K421" s="15" t="inlineStr">
-        <is>
-          <t>enruta</t>
-        </is>
-      </c>
-      <c r="AI421" s="15" t="inlineStr">
-        <is>
-          <t>Ruta: Osorno-LaUnion-RioBueno-Valdivia</t>
-        </is>
-      </c>
-    </row>
-    <row r="422">
-      <c r="A422" s="15" t="inlineStr">
-        <is>
-          <t>20260203</t>
-        </is>
-      </c>
-      <c r="B422" s="15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C422" s="15" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="D422" s="15" t="inlineStr">
-        <is>
-          <t>9999</t>
-        </is>
-      </c>
-      <c r="E422" s="15" t="inlineStr">
-        <is>
-          <t>ACHS OSORNO</t>
-        </is>
-      </c>
-      <c r="F422" s="15" t="inlineStr">
-        <is>
-          <t>Av. Zenteno Nº1529, Osorno</t>
-        </is>
-      </c>
-      <c r="G422" s="15" t="inlineStr">
-        <is>
-          <t>Osorno</t>
-        </is>
-      </c>
-      <c r="H422" s="15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J422" s="15" t="n">
-        <v>10018</v>
-      </c>
-      <c r="K422" s="15" t="inlineStr">
-        <is>
-          <t>enruta</t>
-        </is>
-      </c>
-      <c r="AI422" s="15" t="inlineStr">
-        <is>
-          <t>Ruta: Osorno-LaUnion-RioBueno-Valdivia</t>
-        </is>
-      </c>
-    </row>
-    <row r="423">
-      <c r="A423" s="15" t="inlineStr">
-        <is>
-          <t>20260203</t>
-        </is>
-      </c>
-      <c r="B423" s="15" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="C423" s="15" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="D423" s="15" t="inlineStr">
-        <is>
-          <t>9999</t>
-        </is>
-      </c>
-      <c r="E423" s="15" t="inlineStr">
-        <is>
-          <t>ACHS VALDIVIA</t>
-        </is>
-      </c>
-      <c r="F423" s="15" t="inlineStr">
-        <is>
-          <t>Beauchef Nº705, Valdivia</t>
-        </is>
-      </c>
-      <c r="G423" s="15" t="inlineStr">
-        <is>
-          <t>Valdivia</t>
-        </is>
-      </c>
-      <c r="H423" s="15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J423" s="15" t="n">
-        <v>10036</v>
-      </c>
-      <c r="K423" s="15" t="inlineStr">
-        <is>
-          <t>enruta</t>
-        </is>
-      </c>
-      <c r="AI423" s="15" t="inlineStr">
-        <is>
-          <t>Ruta: Osorno-LaUnion-RioBueno-Valdivia</t>
-        </is>
-      </c>
-    </row>
-    <row r="424">
-      <c r="A424" s="15" t="inlineStr">
-        <is>
-          <t>20260203</t>
-        </is>
-      </c>
-      <c r="B424" s="15" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="C424" s="15" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="D424" s="15" t="inlineStr">
-        <is>
-          <t>77.800.823-8</t>
-        </is>
-      </c>
-      <c r="E424" s="15" t="inlineStr">
-        <is>
-          <t>Clinica Hora Dental</t>
-        </is>
-      </c>
-      <c r="F424" s="15" t="inlineStr">
-        <is>
-          <t>Ramon Picarte 2629</t>
-        </is>
-      </c>
-      <c r="G424" s="15" t="inlineStr">
-        <is>
-          <t>Valdivia</t>
-        </is>
-      </c>
-      <c r="H424" s="15" t="inlineStr">
-        <is>
-          <t>999197935</t>
-        </is>
-      </c>
-      <c r="I424" s="15" t="inlineStr">
-        <is>
-          <t>09:30 a 13:00 y de 15:30 a 19:00</t>
-        </is>
-      </c>
-      <c r="J424" s="15" t="n">
-        <v>10177</v>
-      </c>
-      <c r="K424" s="15" t="inlineStr">
-        <is>
-          <t>enruta</t>
-        </is>
-      </c>
-      <c r="AI424" s="15" t="inlineStr">
-        <is>
-          <t>Ruta: Osorno-LaUnion-RioBueno-Valdivia</t>
-        </is>
-      </c>
-    </row>
-    <row r="425">
-      <c r="A425" s="15" t="inlineStr">
-        <is>
-          <t>20260203</t>
-        </is>
-      </c>
-      <c r="B425" s="15" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="C425" s="15" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="D425" s="15" t="inlineStr">
-        <is>
-          <t>77.512.587-k</t>
-        </is>
-      </c>
-      <c r="E425" s="15" t="inlineStr">
-        <is>
-          <t>maria jo beauty estudio</t>
-        </is>
-      </c>
-      <c r="F425" s="15" t="inlineStr">
-        <is>
-          <t>janequeo 368</t>
-        </is>
-      </c>
-      <c r="G425" s="15" t="inlineStr">
-        <is>
-          <t>Valdivia</t>
-        </is>
-      </c>
-      <c r="H425" s="15" t="inlineStr">
-        <is>
-          <t>972955740</t>
-        </is>
-      </c>
-      <c r="I425" s="15" t="inlineStr">
-        <is>
-          <t>desde las 14:00</t>
-        </is>
-      </c>
-      <c r="J425" s="15" t="n">
-        <v>10175</v>
-      </c>
-      <c r="K425" s="15" t="inlineStr">
-        <is>
-          <t>enruta</t>
-        </is>
-      </c>
-      <c r="AI425" s="15" t="inlineStr">
-        <is>
-          <t>Ruta: Osorno-LaUnion-RioBueno-Valdivia</t>
-        </is>
-      </c>
-    </row>
-    <row r="426">
-      <c r="A426" s="15" t="inlineStr">
-        <is>
-          <t>20260203</t>
-        </is>
-      </c>
-      <c r="B426" s="15" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="C426" s="15" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="D426" s="15" t="inlineStr">
-        <is>
-          <t>77.574.343-3</t>
-        </is>
-      </c>
-      <c r="E426" s="15" t="inlineStr">
-        <is>
-          <t>Odontología y estética Dra Gallardo SpA</t>
-        </is>
-      </c>
-      <c r="F426" s="15" t="inlineStr">
-        <is>
-          <t>Arauco561, OF 706</t>
-        </is>
-      </c>
-      <c r="G426" s="15" t="inlineStr">
-        <is>
-          <t>Valdivia</t>
-        </is>
-      </c>
-      <c r="H426" s="15" t="inlineStr">
-        <is>
-          <t>940553882</t>
-        </is>
-      </c>
-      <c r="I426" s="15" t="inlineStr">
-        <is>
-          <t>10 a 14 y 15 a 19</t>
-        </is>
-      </c>
-      <c r="J426" s="15" t="n">
-        <v>10149</v>
-      </c>
-      <c r="K426" s="15" t="inlineStr">
-        <is>
-          <t>enruta</t>
-        </is>
-      </c>
-      <c r="AI426" s="15" t="inlineStr">
-        <is>
-          <t>Ruta: Osorno-LaUnion-RioBueno-Valdivia</t>
-        </is>
-      </c>
-    </row>
-    <row r="427">
-      <c r="A427" s="15" t="inlineStr">
-        <is>
-          <t>20260203</t>
-        </is>
-      </c>
-      <c r="B427" s="15" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="C427" s="15" t="inlineStr">
-        <is>
-          <t>90</t>
-        </is>
-      </c>
-      <c r="D427" s="15" t="inlineStr">
-        <is>
-          <t>77.018.394-4</t>
-        </is>
-      </c>
-      <c r="E427" s="15" t="inlineStr">
-        <is>
-          <t>Servicios Medicos Limitada</t>
-        </is>
-      </c>
-      <c r="F427" s="15" t="inlineStr">
-        <is>
-          <t>Arauco561, OF 701</t>
-        </is>
-      </c>
-      <c r="G427" s="15" t="inlineStr">
-        <is>
-          <t>Valdivia</t>
-        </is>
-      </c>
-      <c r="H427" s="15" t="inlineStr">
-        <is>
-          <t>966670399</t>
-        </is>
-      </c>
-      <c r="I427" s="15" t="inlineStr">
-        <is>
-          <t>cliente nuevo 1c y 1b / retirar 1c 1lts /14 a 20</t>
-        </is>
-      </c>
-      <c r="J427" s="15" t="n">
-        <v>10187</v>
-      </c>
-      <c r="K427" s="15" t="inlineStr">
-        <is>
-          <t>enruta</t>
-        </is>
-      </c>
-      <c r="AI427" s="15" t="inlineStr">
-        <is>
-          <t>Ruta: Osorno-LaUnion-RioBueno-Valdivia</t>
-        </is>
-      </c>
-    </row>
-    <row r="428">
-      <c r="A428" s="15" t="inlineStr">
-        <is>
-          <t>20260203</t>
-        </is>
-      </c>
-      <c r="B428" s="15" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="C428" s="15" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="D428" s="15" t="inlineStr">
-        <is>
-          <t>6.576.720-1</t>
-        </is>
-      </c>
-      <c r="E428" s="15" t="inlineStr">
-        <is>
-          <t>Maria isabel Moreno Vivanco (medodonta)</t>
-        </is>
-      </c>
-      <c r="F428" s="15" t="inlineStr">
-        <is>
-          <t>Manuel Montt 0253</t>
-        </is>
-      </c>
-      <c r="G428" s="15" t="inlineStr">
-        <is>
-          <t>Valdivia</t>
-        </is>
-      </c>
-      <c r="H428" s="15" t="inlineStr">
-        <is>
-          <t>998295798</t>
-        </is>
-      </c>
-      <c r="I428" s="15" t="inlineStr">
-        <is>
-          <t>14 a 17:30</t>
-        </is>
-      </c>
-      <c r="J428" s="15" t="n">
-        <v>10188</v>
-      </c>
-      <c r="K428" s="15" t="inlineStr">
-        <is>
-          <t>enruta</t>
-        </is>
-      </c>
-      <c r="AI428" s="15" t="inlineStr">
-        <is>
-          <t>Ruta: Osorno-LaUnion-RioBueno-Valdivia</t>
-        </is>
-      </c>
-    </row>
-    <row r="429">
-      <c r="A429" s="15" t="inlineStr">
-        <is>
-          <t>20260203</t>
-        </is>
-      </c>
-      <c r="B429" s="15" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="C429" s="15" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="D429" s="15" t="inlineStr">
-        <is>
-          <t>77.156.579-4</t>
-        </is>
-      </c>
-      <c r="E429" s="15" t="inlineStr">
-        <is>
-          <t>virtos dos spa.</t>
-        </is>
-      </c>
-      <c r="F429" s="15" t="inlineStr">
-        <is>
-          <t>los alamos 1121,block A dep803</t>
-        </is>
-      </c>
-      <c r="G429" s="15" t="inlineStr">
-        <is>
-          <t>Valdivia</t>
-        </is>
-      </c>
-      <c r="H429" s="15" t="inlineStr">
-        <is>
-          <t>998833928</t>
-        </is>
-      </c>
-      <c r="I429" s="15" t="inlineStr">
-        <is>
-          <t>10 a 20</t>
-        </is>
-      </c>
-      <c r="J429" s="15" t="n">
-        <v>10174</v>
-      </c>
-      <c r="K429" s="15" t="inlineStr">
-        <is>
-          <t>enruta</t>
-        </is>
-      </c>
-      <c r="AI429" s="15" t="inlineStr">
-        <is>
-          <t>Ruta: Osorno-LaUnion-RioBueno-Valdivia</t>
-        </is>
-      </c>
-    </row>
-    <row r="430">
-      <c r="A430" s="15" t="inlineStr">
-        <is>
-          <t>20260203</t>
-        </is>
-      </c>
-      <c r="B430" s="15" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="C430" s="15" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="D430" s="15" t="inlineStr">
-        <is>
-          <t>77.149.769-1</t>
-        </is>
-      </c>
-      <c r="E430" s="15" t="inlineStr">
-        <is>
-          <t>Medic Home spa</t>
-        </is>
-      </c>
-      <c r="F430" s="15" t="inlineStr">
-        <is>
-          <t>condominio doña ines , parc 40</t>
-        </is>
-      </c>
-      <c r="G430" s="15" t="inlineStr">
-        <is>
-          <t>Valdivia</t>
-        </is>
-      </c>
-      <c r="H430" s="15" t="inlineStr">
-        <is>
-          <t>988108996</t>
-        </is>
-      </c>
-      <c r="I430" s="15" t="inlineStr">
-        <is>
-          <t>todo el dia</t>
-        </is>
-      </c>
-      <c r="J430" s="15" t="n">
-        <v>10023</v>
-      </c>
-      <c r="K430" s="15" t="inlineStr">
-        <is>
-          <t>enruta</t>
-        </is>
-      </c>
-      <c r="AI430" s="15" t="inlineStr">
-        <is>
-          <t>Ruta: Osorno-LaUnion-RioBueno-Valdivia</t>
-        </is>
-      </c>
-    </row>
-    <row r="431">
-      <c r="A431" s="15" t="inlineStr">
-        <is>
-          <t>20260203</t>
-        </is>
-      </c>
-      <c r="B431" s="15" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="C431" s="15" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="D431" s="15" t="inlineStr">
-        <is>
-          <t>70.362.000-0</t>
-        </is>
-      </c>
-      <c r="E431" s="15" t="inlineStr">
-        <is>
-          <t>Corporación para la nutrición infantil</t>
-        </is>
-      </c>
-      <c r="F431" s="15" t="inlineStr">
-        <is>
-          <t>Ruben Dario 285, El laurel</t>
-        </is>
-      </c>
-      <c r="G431" s="15" t="inlineStr">
-        <is>
-          <t>Valdivia</t>
-        </is>
-      </c>
-      <c r="H431" s="15" t="inlineStr">
-        <is>
-          <t>988612484</t>
-        </is>
-      </c>
-      <c r="I431" s="15" t="inlineStr">
-        <is>
-          <t>con deuda o problema: suspendido desde santiago</t>
-        </is>
-      </c>
-      <c r="J431" s="15" t="n">
-        <v>10147</v>
-      </c>
-      <c r="K431" s="15" t="inlineStr">
-        <is>
-          <t>enruta</t>
-        </is>
-      </c>
-      <c r="AI431" s="15" t="inlineStr">
-        <is>
-          <t>Ruta: Osorno-LaUnion-RioBueno-Valdivia</t>
-        </is>
-      </c>
-    </row>
-    <row r="432">
-      <c r="A432" s="15" t="inlineStr">
-        <is>
-          <t>20260203</t>
-        </is>
-      </c>
-      <c r="B432" s="15" t="n">
-        <v>23</v>
-      </c>
-      <c r="C432" s="15" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="D432" s="15" t="inlineStr">
-        <is>
-          <t>77.874.165-4</t>
-        </is>
-      </c>
-      <c r="E432" s="15" t="inlineStr">
-        <is>
-          <t>centro medico veterinario Reloncavi spa</t>
-        </is>
-      </c>
-      <c r="F432" s="15" t="inlineStr">
-        <is>
-          <t>serrano 27</t>
-        </is>
-      </c>
-      <c r="G432" s="15" t="inlineStr">
-        <is>
-          <t>Puerto Montt</t>
-        </is>
-      </c>
-      <c r="H432" s="15" t="inlineStr">
-        <is>
-          <t>977745392/921776772</t>
-        </is>
-      </c>
-      <c r="I432" s="15" t="inlineStr">
-        <is>
-          <t>cliente ingresado automaticamente</t>
-        </is>
-      </c>
-      <c r="J432" s="15" t="n">
-        <v>10062</v>
-      </c>
-      <c r="K432" s="15" t="inlineStr">
-        <is>
-          <t>REALIZADO</t>
-        </is>
-      </c>
-      <c r="L432" s="15" t="inlineStr">
-        <is>
-          <t>ca3l10 ba10 mensaje extra</t>
-        </is>
-      </c>
-      <c r="Z432" s="15" t="n">
-        <v>10</v>
-      </c>
-      <c r="AF432" s="15" t="n">
-        <v>10</v>
-      </c>
-      <c r="AI432" s="15" t="inlineStr">
-        <is>
-          <t>Ruta: Osorno-LaUnion-RioBueno-Valdivia</t>
         </is>
       </c>
     </row>
@@ -41740,7 +40159,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E93"/>
+  <dimension ref="A1:E95"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.5859375" defaultRowHeight="13.8" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9.48" customWidth="1" style="23" min="1" max="1"/>
@@ -41833,7 +40252,7 @@
       </c>
       <c r="D4" s="23" t="inlineStr">
         <is>
-          <t>vigente</t>
+          <t>rendido</t>
         </is>
       </c>
     </row>
@@ -41851,15 +40270,58 @@
       </c>
       <c r="D5" s="23" t="inlineStr">
         <is>
-          <t>vigente</t>
+          <t>rendido</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="16">
-      <c r="C6" s="24" t="n"/>
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>20251012</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>-5000</t>
+        </is>
+      </c>
+      <c r="C6" s="24" t="inlineStr">
+        <is>
+          <t>estacionamiento prueba</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>rendido</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="16">
-      <c r="C7" s="24" t="n"/>
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>20251031</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>-5000</t>
+        </is>
+      </c>
+      <c r="C7" s="24" t="inlineStr">
+        <is>
+          <t>prueba</t>
+        </is>
+      </c>
+      <c r="D7" s="15" t="inlineStr">
+        <is>
+          <t>rendido</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="16">
       <c r="C8" s="24" t="n"/>
@@ -42119,8 +40581,12 @@
     <row r="93" ht="15.75" customHeight="1" s="16">
       <c r="C93" s="24" t="n"/>
     </row>
-    <row r="94" ht="15.75" customHeight="1" s="16"/>
-    <row r="95" ht="15.75" customHeight="1" s="16"/>
+    <row r="94" ht="15.75" customHeight="1" s="16">
+      <c r="C94" s="24" t="n"/>
+    </row>
+    <row r="95" ht="15.75" customHeight="1" s="16">
+      <c r="C95" s="24" t="n"/>
+    </row>
     <row r="96" ht="15.75" customHeight="1" s="16"/>
     <row r="97" ht="15.75" customHeight="1" s="16"/>
     <row r="98" ht="15.75" customHeight="1" s="16"/>
@@ -42147,7 +40613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:X273"/>
+  <dimension ref="A1:X271"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.5859375" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8" customWidth="1" style="15" min="1" max="24"/>
@@ -42285,34 +40751,34 @@
         <v>0</v>
       </c>
       <c r="G2" s="15" t="n">
-        <v>0</v>
+        <v>-25</v>
       </c>
       <c r="H2" s="15" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I2" s="15" t="n">
         <v>0</v>
       </c>
       <c r="J2" s="15" t="n">
-        <v>80</v>
+        <v>10</v>
       </c>
       <c r="K2" s="15" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="L2" s="15" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="M2" s="15" t="n">
         <v>0</v>
       </c>
       <c r="N2" s="15" t="n">
-        <v>0</v>
+        <v>54</v>
       </c>
       <c r="O2" s="15" t="n">
         <v>0</v>
       </c>
       <c r="P2" s="15" t="n">
-        <v>80</v>
+        <v>161</v>
       </c>
       <c r="Q2" s="15" t="n">
         <v>0</v>
@@ -42327,16 +40793,80 @@
         <v>0</v>
       </c>
       <c r="U2" s="15" t="n">
+        <v>35</v>
+      </c>
+      <c r="V2" s="15" t="n">
+        <v>150</v>
+      </c>
+      <c r="W2" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" ht="13.5" customHeight="1" s="16">
+      <c r="C3" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="V2" s="15" t="n">
+      <c r="D3" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="W2" s="15" t="n">
+      <c r="E3" s="15" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" ht="13.5" customHeight="1" s="16"/>
+      <c r="F3" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="V3" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="W3" t="n">
+        <v>0</v>
+      </c>
+    </row>
     <row r="4" ht="13.5" customHeight="1" s="16">
       <c r="A4" s="15" t="inlineStr">
         <is>
@@ -46091,54 +44621,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="271">
-      <c r="A271" s="15" t="inlineStr">
-        <is>
-          <t>20260203</t>
-        </is>
-      </c>
-      <c r="B271" s="15" t="n">
-        <v>10017</v>
-      </c>
-      <c r="J271" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="P271" s="15" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="272">
-      <c r="A272" s="15" t="inlineStr">
-        <is>
-          <t>20260203</t>
-        </is>
-      </c>
-      <c r="B272" s="15" t="n">
-        <v>10016</v>
-      </c>
-      <c r="J272" s="15" t="n">
-        <v>10</v>
-      </c>
-      <c r="P272" s="15" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="273">
-      <c r="A273" s="15" t="inlineStr">
-        <is>
-          <t>20260203</t>
-        </is>
-      </c>
-      <c r="B273" s="15" t="n">
-        <v>10062</v>
-      </c>
-      <c r="J273" s="15" t="n">
-        <v>10</v>
-      </c>
-      <c r="P273" s="15" t="n">
-        <v>10</v>
-      </c>
-    </row>
+    <row r="271"/>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0" footer="0"/>

</xml_diff>

<commit_message>
Trabajando en nueva ruta y estilos
Trabajando en estilo de tarjetas, y en nueva ruta visualizadora
</commit_message>
<xml_diff>
--- a/bd/mediclean_bd.xlsx
+++ b/bd/mediclean_bd.xlsx
@@ -615,7 +615,7 @@
       </c>
       <c r="C2" s="17" t="inlineStr">
         <is>
-          <t>2XJTmILSBd_seuuDlxm478aVSZ1gOUBx0M0nfZNbAQ0</t>
+          <t>1rn8seeBVIH7e0-90mCWIuz8esKnvnMEnXWttJXOt78</t>
         </is>
       </c>
     </row>
@@ -42160,7 +42160,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:X277"/>
+  <dimension ref="A1:X276"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.59375" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8" customWidth="1" style="14" min="1" max="24"/>
@@ -46255,7 +46255,6 @@
         <v>2</v>
       </c>
     </row>
-    <row r="277"/>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0" footer="0"/>

</xml_diff>

<commit_message>
Corrigiendo error en boton eliminar item de rutaactual
</commit_message>
<xml_diff>
--- a/bd/mediclean_bd.xlsx
+++ b/bd/mediclean_bd.xlsx
@@ -615,7 +615,7 @@
       </c>
       <c r="C2" s="17" t="inlineStr">
         <is>
-          <t>1rn8seeBVIH7e0-90mCWIuz8esKnvnMEnXWttJXOt78</t>
+          <t>Aqa1XLWSxZtU1jzgz9xIzrrYT5KxIkvADqR9yiSP4CQ</t>
         </is>
       </c>
     </row>
@@ -11425,7 +11425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AN432"/>
+  <dimension ref="A1:AN431"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.59375" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8.699999999999999" customWidth="1" style="14" min="1" max="1"/>
@@ -40473,27 +40473,27 @@
       </c>
       <c r="B412" s="14" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C412" s="14" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>30</t>
         </is>
       </c>
       <c r="D412" s="14" t="inlineStr">
         <is>
-          <t>77.141.505-9</t>
+          <t>76.828.443-1</t>
         </is>
       </c>
       <c r="E412" s="14" t="inlineStr">
         <is>
-          <t>centro odont. Familiar Ultradens</t>
+          <t>Servicios Odontologicos CRD SpA</t>
         </is>
       </c>
       <c r="F412" s="14" t="inlineStr">
         <is>
-          <t>Ramirez 684</t>
+          <t>Pasaje Consistorial, local K</t>
         </is>
       </c>
       <c r="G412" s="14" t="inlineStr">
@@ -40503,29 +40503,29 @@
       </c>
       <c r="H412" s="14" t="inlineStr">
         <is>
-          <t>933892771</t>
+          <t>998422751</t>
         </is>
       </c>
       <c r="I412" s="14" t="inlineStr">
         <is>
-          <t>9:30 a 13 y 15 a 19</t>
+          <t>10 A 14 Y 15 A 20</t>
         </is>
       </c>
       <c r="J412" s="14" t="n">
-        <v>10112</v>
+        <v>10014</v>
       </c>
       <c r="K412" s="14" t="inlineStr">
         <is>
-          <t>enruta</t>
+          <t>REALIZADO</t>
         </is>
       </c>
       <c r="L412" s="14" t="inlineStr">
         <is>
-          <t>ca3l8</t>
+          <t>ca3l2</t>
         </is>
       </c>
       <c r="Z412" s="14" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="AI412" s="14" t="inlineStr">
         <is>
@@ -40541,27 +40541,27 @@
       </c>
       <c r="B413" s="14" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C413" s="14" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>60</t>
         </is>
       </c>
       <c r="D413" s="14" t="inlineStr">
         <is>
-          <t>76.828.443-1</t>
+          <t>76.792.132-2</t>
         </is>
       </c>
       <c r="E413" s="14" t="inlineStr">
         <is>
-          <t>Servicios Odontologicos CRD SpA</t>
+          <t>Giacomozzi y Paves ltda</t>
         </is>
       </c>
       <c r="F413" s="14" t="inlineStr">
         <is>
-          <t>Pasaje Consistorial, local K</t>
+          <t>Gillermo buhler 1561</t>
         </is>
       </c>
       <c r="G413" s="14" t="inlineStr">
@@ -40571,29 +40571,21 @@
       </c>
       <c r="H413" s="14" t="inlineStr">
         <is>
-          <t>998422751</t>
+          <t>977491966/952115168</t>
         </is>
       </c>
       <c r="I413" s="14" t="inlineStr">
         <is>
-          <t>10 A 14 Y 15 A 20</t>
+          <t>ultimo retiro febrero 2025</t>
         </is>
       </c>
       <c r="J413" s="14" t="n">
-        <v>10014</v>
+        <v>10035</v>
       </c>
       <c r="K413" s="14" t="inlineStr">
         <is>
-          <t>REALIZADO</t>
-        </is>
-      </c>
-      <c r="L413" s="14" t="inlineStr">
-        <is>
-          <t>ca3l2</t>
-        </is>
-      </c>
-      <c r="Z413" s="14" t="n">
-        <v>2</v>
+          <t>enruta</t>
+        </is>
       </c>
       <c r="AI413" s="14" t="inlineStr">
         <is>
@@ -40609,7 +40601,7 @@
       </c>
       <c r="B414" s="14" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C414" s="14" t="inlineStr">
@@ -40619,17 +40611,17 @@
       </c>
       <c r="D414" s="14" t="inlineStr">
         <is>
-          <t>76.958.988-0</t>
+          <t>65.104.083-3</t>
         </is>
       </c>
       <c r="E414" s="14" t="inlineStr">
         <is>
-          <t>clinica veterinaria Mundo animal</t>
+          <t>Fundacion Proseger, Servicio Geriatrico</t>
         </is>
       </c>
       <c r="F414" s="14" t="inlineStr">
         <is>
-          <t>Zenteno 2748</t>
+          <t>Mackenna 1040</t>
         </is>
       </c>
       <c r="G414" s="14" t="inlineStr">
@@ -40639,20 +40631,25 @@
       </c>
       <c r="H414" s="14" t="inlineStr">
         <is>
-          <t>6442264990/990004454</t>
+          <t>642481595</t>
         </is>
       </c>
       <c r="I414" s="14" t="inlineStr">
         <is>
-          <t>10 a 14 y 15 a 19/ monserrat</t>
+          <t>con deuda o problema</t>
         </is>
       </c>
       <c r="J414" s="14" t="n">
-        <v>10015</v>
+        <v>10019</v>
       </c>
       <c r="K414" s="14" t="inlineStr">
         <is>
-          <t>enruta</t>
+          <t>POSPUESTO</t>
+        </is>
+      </c>
+      <c r="L414" s="14" t="inlineStr">
+        <is>
+          <t>con deuda o problema</t>
         </is>
       </c>
       <c r="AI414" s="14" t="inlineStr">
@@ -40669,7 +40666,7 @@
       </c>
       <c r="B415" s="14" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C415" s="14" t="inlineStr">
@@ -40679,17 +40676,17 @@
       </c>
       <c r="D415" s="14" t="inlineStr">
         <is>
-          <t>76.792.132-2</t>
+          <t>77.884.397-8</t>
         </is>
       </c>
       <c r="E415" s="14" t="inlineStr">
         <is>
-          <t>Giacomozzi y Paves ltda</t>
+          <t>centro odontologico carvajal y fernandez ltda</t>
         </is>
       </c>
       <c r="F415" s="14" t="inlineStr">
         <is>
-          <t>Gillermo buhler 1561</t>
+          <t>o´higgins 485 of 408</t>
         </is>
       </c>
       <c r="G415" s="14" t="inlineStr">
@@ -40699,16 +40696,16 @@
       </c>
       <c r="H415" s="14" t="inlineStr">
         <is>
-          <t>977491966/952115168</t>
+          <t>975643988/971381140</t>
         </is>
       </c>
       <c r="I415" s="14" t="inlineStr">
         <is>
-          <t>ultimo retiro febrero 2025</t>
+          <t>con deuda o problema</t>
         </is>
       </c>
       <c r="J415" s="14" t="n">
-        <v>10035</v>
+        <v>10185</v>
       </c>
       <c r="K415" s="14" t="inlineStr">
         <is>
@@ -40729,7 +40726,7 @@
       </c>
       <c r="B416" s="14" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>11</t>
         </is>
       </c>
       <c r="C416" s="14" t="inlineStr">
@@ -40739,45 +40736,40 @@
       </c>
       <c r="D416" s="14" t="inlineStr">
         <is>
-          <t>65.104.083-3</t>
+          <t>77.016.887-2</t>
         </is>
       </c>
       <c r="E416" s="14" t="inlineStr">
         <is>
-          <t>Fundacion Proseger, Servicio Geriatrico</t>
+          <t>Oro.odontologia especializada dra natalia marti</t>
         </is>
       </c>
       <c r="F416" s="14" t="inlineStr">
         <is>
-          <t>Mackenna 1040</t>
+          <t>arturo prat 662</t>
         </is>
       </c>
       <c r="G416" s="14" t="inlineStr">
         <is>
-          <t>Osorno</t>
+          <t>La Union</t>
         </is>
       </c>
       <c r="H416" s="14" t="inlineStr">
         <is>
-          <t>642481595</t>
+          <t>972698736</t>
         </is>
       </c>
       <c r="I416" s="14" t="inlineStr">
         <is>
-          <t>con deuda o problema</t>
+          <t>10 a 13:30 y 15 a 19:30</t>
         </is>
       </c>
       <c r="J416" s="14" t="n">
-        <v>10019</v>
+        <v>10186</v>
       </c>
       <c r="K416" s="14" t="inlineStr">
         <is>
-          <t>POSPUESTO</t>
-        </is>
-      </c>
-      <c r="L416" s="14" t="inlineStr">
-        <is>
-          <t>con deuda o problema</t>
+          <t>enruta</t>
         </is>
       </c>
       <c r="AI416" s="14" t="inlineStr">
@@ -40794,46 +40786,46 @@
       </c>
       <c r="B417" s="14" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C417" s="14" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>30</t>
         </is>
       </c>
       <c r="D417" s="14" t="inlineStr">
         <is>
-          <t>77.884.397-8</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="E417" s="14" t="inlineStr">
         <is>
-          <t>centro odontologico carvajal y fernandez ltda</t>
+          <t>ACHS LA UNION</t>
         </is>
       </c>
       <c r="F417" s="14" t="inlineStr">
         <is>
-          <t>o´higgins 485 of 408</t>
+          <t>Comercio Nº260, La Unión</t>
         </is>
       </c>
       <c r="G417" s="14" t="inlineStr">
         <is>
-          <t>Osorno</t>
+          <t>La Union</t>
         </is>
       </c>
       <c r="H417" s="14" t="inlineStr">
         <is>
-          <t>975643988/971381140</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I417" s="14" t="inlineStr">
         <is>
-          <t>con deuda o problema</t>
+          <t>con deuda o problema: EN REMODELACION</t>
         </is>
       </c>
       <c r="J417" s="14" t="n">
-        <v>10185</v>
+        <v>10020</v>
       </c>
       <c r="K417" s="14" t="inlineStr">
         <is>
@@ -40854,46 +40846,41 @@
       </c>
       <c r="B418" s="14" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C418" s="14" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>30</t>
         </is>
       </c>
       <c r="D418" s="14" t="inlineStr">
         <is>
-          <t>77.016.887-2</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="E418" s="14" t="inlineStr">
         <is>
-          <t>Oro.odontologia especializada dra natalia marti</t>
+          <t>ACHS Rio Bueno</t>
         </is>
       </c>
       <c r="F418" s="14" t="inlineStr">
         <is>
-          <t>arturo prat 662</t>
+          <t>Independencia Nº970</t>
         </is>
       </c>
       <c r="G418" s="14" t="inlineStr">
         <is>
-          <t>La Union</t>
+          <t>Rio bueno</t>
         </is>
       </c>
       <c r="H418" s="14" t="inlineStr">
         <is>
-          <t>972698736</t>
-        </is>
-      </c>
-      <c r="I418" s="14" t="inlineStr">
-        <is>
-          <t>10 a 13:30 y 15 a 19:30</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J418" s="14" t="n">
-        <v>10186</v>
+        <v>10021</v>
       </c>
       <c r="K418" s="14" t="inlineStr">
         <is>
@@ -40914,46 +40901,46 @@
       </c>
       <c r="B419" s="14" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>13</t>
         </is>
       </c>
       <c r="C419" s="14" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>60</t>
         </is>
       </c>
       <c r="D419" s="14" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>77.574.343-3</t>
         </is>
       </c>
       <c r="E419" s="14" t="inlineStr">
         <is>
-          <t>ACHS LA UNION</t>
+          <t>Odontología y estética Dra Gallardo SpA</t>
         </is>
       </c>
       <c r="F419" s="14" t="inlineStr">
         <is>
-          <t>Comercio Nº260, La Unión</t>
+          <t>San Martín 1465</t>
         </is>
       </c>
       <c r="G419" s="14" t="inlineStr">
         <is>
-          <t>La Union</t>
+          <t>Rio bueno</t>
         </is>
       </c>
       <c r="H419" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>940553882</t>
         </is>
       </c>
       <c r="I419" s="14" t="inlineStr">
         <is>
-          <t>con deuda o problema: EN REMODELACION</t>
+          <t>10 a 14 y 15 a 19</t>
         </is>
       </c>
       <c r="J419" s="14" t="n">
-        <v>10020</v>
+        <v>10149</v>
       </c>
       <c r="K419" s="14" t="inlineStr">
         <is>
@@ -40974,12 +40961,12 @@
       </c>
       <c r="B420" s="14" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C420" s="14" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>15</t>
         </is>
       </c>
       <c r="D420" s="14" t="inlineStr">
@@ -40989,17 +40976,17 @@
       </c>
       <c r="E420" s="14" t="inlineStr">
         <is>
-          <t>ACHS Rio Bueno</t>
+          <t>ACHS OSORNO</t>
         </is>
       </c>
       <c r="F420" s="14" t="inlineStr">
         <is>
-          <t>Independencia Nº970</t>
+          <t>Av. Zenteno Nº1529, Osorno</t>
         </is>
       </c>
       <c r="G420" s="14" t="inlineStr">
         <is>
-          <t>Rio bueno</t>
+          <t>Osorno</t>
         </is>
       </c>
       <c r="H420" s="14" t="inlineStr">
@@ -41008,7 +40995,7 @@
         </is>
       </c>
       <c r="J420" s="14" t="n">
-        <v>10021</v>
+        <v>10018</v>
       </c>
       <c r="K420" s="14" t="inlineStr">
         <is>
@@ -41029,46 +41016,41 @@
       </c>
       <c r="B421" s="14" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C421" s="14" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>15</t>
         </is>
       </c>
       <c r="D421" s="14" t="inlineStr">
         <is>
-          <t>77.574.343-3</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="E421" s="14" t="inlineStr">
         <is>
-          <t>Odontología y estética Dra Gallardo SpA</t>
+          <t>ACHS VALDIVIA</t>
         </is>
       </c>
       <c r="F421" s="14" t="inlineStr">
         <is>
-          <t>San Martín 1465</t>
+          <t>Beauchef Nº705, Valdivia</t>
         </is>
       </c>
       <c r="G421" s="14" t="inlineStr">
         <is>
-          <t>Rio bueno</t>
+          <t>Valdivia</t>
         </is>
       </c>
       <c r="H421" s="14" t="inlineStr">
         <is>
-          <t>940553882</t>
-        </is>
-      </c>
-      <c r="I421" s="14" t="inlineStr">
-        <is>
-          <t>10 a 14 y 15 a 19</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J421" s="14" t="n">
-        <v>10149</v>
+        <v>10036</v>
       </c>
       <c r="K421" s="14" t="inlineStr">
         <is>
@@ -41089,41 +41071,46 @@
       </c>
       <c r="B422" s="14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C422" s="14" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>60</t>
         </is>
       </c>
       <c r="D422" s="14" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>77.800.823-8</t>
         </is>
       </c>
       <c r="E422" s="14" t="inlineStr">
         <is>
-          <t>ACHS OSORNO</t>
+          <t>Clinica Hora Dental</t>
         </is>
       </c>
       <c r="F422" s="14" t="inlineStr">
         <is>
-          <t>Av. Zenteno Nº1529, Osorno</t>
+          <t>Ramon Picarte 2629</t>
         </is>
       </c>
       <c r="G422" s="14" t="inlineStr">
         <is>
-          <t>Osorno</t>
+          <t>Valdivia</t>
         </is>
       </c>
       <c r="H422" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>999197935</t>
+        </is>
+      </c>
+      <c r="I422" s="14" t="inlineStr">
+        <is>
+          <t>09:30 a 13:00 y de 15:30 a 19:00</t>
         </is>
       </c>
       <c r="J422" s="14" t="n">
-        <v>10018</v>
+        <v>10177</v>
       </c>
       <c r="K422" s="14" t="inlineStr">
         <is>
@@ -41144,27 +41131,27 @@
       </c>
       <c r="B423" s="14" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>21</t>
         </is>
       </c>
       <c r="C423" s="14" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>60</t>
         </is>
       </c>
       <c r="D423" s="14" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>77.512.587-k</t>
         </is>
       </c>
       <c r="E423" s="14" t="inlineStr">
         <is>
-          <t>ACHS VALDIVIA</t>
+          <t>maria jo beauty estudio</t>
         </is>
       </c>
       <c r="F423" s="14" t="inlineStr">
         <is>
-          <t>Beauchef Nº705, Valdivia</t>
+          <t>janequeo 368</t>
         </is>
       </c>
       <c r="G423" s="14" t="inlineStr">
@@ -41174,11 +41161,16 @@
       </c>
       <c r="H423" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>972955740</t>
+        </is>
+      </c>
+      <c r="I423" s="14" t="inlineStr">
+        <is>
+          <t>desde las 14:00</t>
         </is>
       </c>
       <c r="J423" s="14" t="n">
-        <v>10036</v>
+        <v>10175</v>
       </c>
       <c r="K423" s="14" t="inlineStr">
         <is>
@@ -41199,7 +41191,7 @@
       </c>
       <c r="B424" s="14" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>14</t>
         </is>
       </c>
       <c r="C424" s="14" t="inlineStr">
@@ -41209,17 +41201,17 @@
       </c>
       <c r="D424" s="14" t="inlineStr">
         <is>
-          <t>77.800.823-8</t>
+          <t>77.574.343-3</t>
         </is>
       </c>
       <c r="E424" s="14" t="inlineStr">
         <is>
-          <t>Clinica Hora Dental</t>
+          <t>Odontología y estética Dra Gallardo SpA</t>
         </is>
       </c>
       <c r="F424" s="14" t="inlineStr">
         <is>
-          <t>Ramon Picarte 2629</t>
+          <t>Arauco561, OF 706</t>
         </is>
       </c>
       <c r="G424" s="14" t="inlineStr">
@@ -41229,16 +41221,16 @@
       </c>
       <c r="H424" s="14" t="inlineStr">
         <is>
-          <t>999197935</t>
+          <t>940553882</t>
         </is>
       </c>
       <c r="I424" s="14" t="inlineStr">
         <is>
-          <t>09:30 a 13:00 y de 15:30 a 19:00</t>
+          <t>10 a 14 y 15 a 19</t>
         </is>
       </c>
       <c r="J424" s="14" t="n">
-        <v>10177</v>
+        <v>10149</v>
       </c>
       <c r="K424" s="14" t="inlineStr">
         <is>
@@ -41259,27 +41251,27 @@
       </c>
       <c r="B425" s="14" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C425" s="14" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>90</t>
         </is>
       </c>
       <c r="D425" s="14" t="inlineStr">
         <is>
-          <t>77.512.587-k</t>
+          <t>77.018.394-4</t>
         </is>
       </c>
       <c r="E425" s="14" t="inlineStr">
         <is>
-          <t>maria jo beauty estudio</t>
+          <t>Servicios Medicos Limitada</t>
         </is>
       </c>
       <c r="F425" s="14" t="inlineStr">
         <is>
-          <t>janequeo 368</t>
+          <t>Arauco561, OF 701</t>
         </is>
       </c>
       <c r="G425" s="14" t="inlineStr">
@@ -41289,16 +41281,16 @@
       </c>
       <c r="H425" s="14" t="inlineStr">
         <is>
-          <t>972955740</t>
+          <t>966670399</t>
         </is>
       </c>
       <c r="I425" s="14" t="inlineStr">
         <is>
-          <t>desde las 14:00</t>
+          <t>cliente nuevo 1c y 1b / retirar 1c 1lts /14 a 20</t>
         </is>
       </c>
       <c r="J425" s="14" t="n">
-        <v>10175</v>
+        <v>10187</v>
       </c>
       <c r="K425" s="14" t="inlineStr">
         <is>
@@ -41319,7 +41311,7 @@
       </c>
       <c r="B426" s="14" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>22</t>
         </is>
       </c>
       <c r="C426" s="14" t="inlineStr">
@@ -41329,17 +41321,17 @@
       </c>
       <c r="D426" s="14" t="inlineStr">
         <is>
-          <t>77.574.343-3</t>
+          <t>6.576.720-1</t>
         </is>
       </c>
       <c r="E426" s="14" t="inlineStr">
         <is>
-          <t>Odontología y estética Dra Gallardo SpA</t>
+          <t>Maria isabel Moreno Vivanco (medodonta)</t>
         </is>
       </c>
       <c r="F426" s="14" t="inlineStr">
         <is>
-          <t>Arauco561, OF 706</t>
+          <t>Manuel Montt 0253</t>
         </is>
       </c>
       <c r="G426" s="14" t="inlineStr">
@@ -41349,16 +41341,16 @@
       </c>
       <c r="H426" s="14" t="inlineStr">
         <is>
-          <t>940553882</t>
+          <t>998295798</t>
         </is>
       </c>
       <c r="I426" s="14" t="inlineStr">
         <is>
-          <t>10 a 14 y 15 a 19</t>
+          <t>14 a 17:30</t>
         </is>
       </c>
       <c r="J426" s="14" t="n">
-        <v>10149</v>
+        <v>10188</v>
       </c>
       <c r="K426" s="14" t="inlineStr">
         <is>
@@ -41379,27 +41371,27 @@
       </c>
       <c r="B427" s="14" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C427" s="14" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>30</t>
         </is>
       </c>
       <c r="D427" s="14" t="inlineStr">
         <is>
-          <t>77.018.394-4</t>
+          <t>77.156.579-4</t>
         </is>
       </c>
       <c r="E427" s="14" t="inlineStr">
         <is>
-          <t>Servicios Medicos Limitada</t>
+          <t>virtos dos spa.</t>
         </is>
       </c>
       <c r="F427" s="14" t="inlineStr">
         <is>
-          <t>Arauco561, OF 701</t>
+          <t>los alamos 1121,block A dep803</t>
         </is>
       </c>
       <c r="G427" s="14" t="inlineStr">
@@ -41409,16 +41401,16 @@
       </c>
       <c r="H427" s="14" t="inlineStr">
         <is>
-          <t>966670399</t>
+          <t>998833928</t>
         </is>
       </c>
       <c r="I427" s="14" t="inlineStr">
         <is>
-          <t>cliente nuevo 1c y 1b / retirar 1c 1lts /14 a 20</t>
+          <t>10 a 20</t>
         </is>
       </c>
       <c r="J427" s="14" t="n">
-        <v>10187</v>
+        <v>10174</v>
       </c>
       <c r="K427" s="14" t="inlineStr">
         <is>
@@ -41439,27 +41431,27 @@
       </c>
       <c r="B428" s="14" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C428" s="14" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>30</t>
         </is>
       </c>
       <c r="D428" s="14" t="inlineStr">
         <is>
-          <t>6.576.720-1</t>
+          <t>77.149.769-1</t>
         </is>
       </c>
       <c r="E428" s="14" t="inlineStr">
         <is>
-          <t>Maria isabel Moreno Vivanco (medodonta)</t>
+          <t>Medic Home spa</t>
         </is>
       </c>
       <c r="F428" s="14" t="inlineStr">
         <is>
-          <t>Manuel Montt 0253</t>
+          <t>condominio doña ines , parc 40</t>
         </is>
       </c>
       <c r="G428" s="14" t="inlineStr">
@@ -41469,16 +41461,16 @@
       </c>
       <c r="H428" s="14" t="inlineStr">
         <is>
-          <t>998295798</t>
+          <t>988108996</t>
         </is>
       </c>
       <c r="I428" s="14" t="inlineStr">
         <is>
-          <t>14 a 17:30</t>
+          <t>todo el dia</t>
         </is>
       </c>
       <c r="J428" s="14" t="n">
-        <v>10188</v>
+        <v>10023</v>
       </c>
       <c r="K428" s="14" t="inlineStr">
         <is>
@@ -41499,7 +41491,7 @@
       </c>
       <c r="B429" s="14" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>19</t>
         </is>
       </c>
       <c r="C429" s="14" t="inlineStr">
@@ -41509,17 +41501,17 @@
       </c>
       <c r="D429" s="14" t="inlineStr">
         <is>
-          <t>77.156.579-4</t>
+          <t>70.362.000-0</t>
         </is>
       </c>
       <c r="E429" s="14" t="inlineStr">
         <is>
-          <t>virtos dos spa.</t>
+          <t>Corporación para la nutrición infantil</t>
         </is>
       </c>
       <c r="F429" s="14" t="inlineStr">
         <is>
-          <t>los alamos 1121,block A dep803</t>
+          <t>Ruben Dario 285, El laurel</t>
         </is>
       </c>
       <c r="G429" s="14" t="inlineStr">
@@ -41529,16 +41521,16 @@
       </c>
       <c r="H429" s="14" t="inlineStr">
         <is>
-          <t>998833928</t>
+          <t>988612484</t>
         </is>
       </c>
       <c r="I429" s="14" t="inlineStr">
         <is>
-          <t>10 a 20</t>
+          <t>con deuda o problema: suspendido desde santiago</t>
         </is>
       </c>
       <c r="J429" s="14" t="n">
-        <v>10174</v>
+        <v>10147</v>
       </c>
       <c r="K429" s="14" t="inlineStr">
         <is>
@@ -41557,53 +41549,62 @@
           <t>20260203</t>
         </is>
       </c>
-      <c r="B430" s="14" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
+      <c r="B430" s="14" t="n">
+        <v>23</v>
       </c>
       <c r="C430" s="14" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>60</t>
         </is>
       </c>
       <c r="D430" s="14" t="inlineStr">
         <is>
-          <t>77.149.769-1</t>
+          <t>77.874.165-4</t>
         </is>
       </c>
       <c r="E430" s="14" t="inlineStr">
         <is>
-          <t>Medic Home spa</t>
+          <t>centro medico veterinario Reloncavi spa</t>
         </is>
       </c>
       <c r="F430" s="14" t="inlineStr">
         <is>
-          <t>condominio doña ines , parc 40</t>
+          <t>serrano 27</t>
         </is>
       </c>
       <c r="G430" s="14" t="inlineStr">
         <is>
-          <t>Valdivia</t>
+          <t>Puerto Montt</t>
         </is>
       </c>
       <c r="H430" s="14" t="inlineStr">
         <is>
-          <t>988108996</t>
+          <t>977745392/921776772</t>
         </is>
       </c>
       <c r="I430" s="14" t="inlineStr">
         <is>
-          <t>todo el dia</t>
+          <t>cliente ingresado automaticamente</t>
         </is>
       </c>
       <c r="J430" s="14" t="n">
-        <v>10023</v>
+        <v>10062</v>
       </c>
       <c r="K430" s="14" t="inlineStr">
         <is>
-          <t>enruta</t>
-        </is>
+          <t>REALIZADO</t>
+        </is>
+      </c>
+      <c r="L430" s="14" t="inlineStr">
+        <is>
+          <t>ca3l10 ba10 mensaje extra</t>
+        </is>
+      </c>
+      <c r="Z430" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="AF430" s="14" t="n">
+        <v>10</v>
       </c>
       <c r="AI430" s="14" t="inlineStr">
         <is>
@@ -41611,135 +41612,8 @@
         </is>
       </c>
     </row>
-    <row r="431" ht="15" customHeight="1" s="15">
-      <c r="A431" s="14" t="inlineStr">
-        <is>
-          <t>20260203</t>
-        </is>
-      </c>
-      <c r="B431" s="14" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="C431" s="14" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="D431" s="14" t="inlineStr">
-        <is>
-          <t>70.362.000-0</t>
-        </is>
-      </c>
-      <c r="E431" s="14" t="inlineStr">
-        <is>
-          <t>Corporación para la nutrición infantil</t>
-        </is>
-      </c>
-      <c r="F431" s="14" t="inlineStr">
-        <is>
-          <t>Ruben Dario 285, El laurel</t>
-        </is>
-      </c>
-      <c r="G431" s="14" t="inlineStr">
-        <is>
-          <t>Valdivia</t>
-        </is>
-      </c>
-      <c r="H431" s="14" t="inlineStr">
-        <is>
-          <t>988612484</t>
-        </is>
-      </c>
-      <c r="I431" s="14" t="inlineStr">
-        <is>
-          <t>con deuda o problema: suspendido desde santiago</t>
-        </is>
-      </c>
-      <c r="J431" s="14" t="n">
-        <v>10147</v>
-      </c>
-      <c r="K431" s="14" t="inlineStr">
-        <is>
-          <t>enruta</t>
-        </is>
-      </c>
-      <c r="AI431" s="14" t="inlineStr">
-        <is>
-          <t>Ruta: Osorno-LaUnion-RioBueno-Valdivia</t>
-        </is>
-      </c>
-    </row>
-    <row r="432" ht="15" customHeight="1" s="15">
-      <c r="A432" s="14" t="inlineStr">
-        <is>
-          <t>20260203</t>
-        </is>
-      </c>
-      <c r="B432" s="14" t="n">
-        <v>23</v>
-      </c>
-      <c r="C432" s="14" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="D432" s="14" t="inlineStr">
-        <is>
-          <t>77.874.165-4</t>
-        </is>
-      </c>
-      <c r="E432" s="14" t="inlineStr">
-        <is>
-          <t>centro medico veterinario Reloncavi spa</t>
-        </is>
-      </c>
-      <c r="F432" s="14" t="inlineStr">
-        <is>
-          <t>serrano 27</t>
-        </is>
-      </c>
-      <c r="G432" s="14" t="inlineStr">
-        <is>
-          <t>Puerto Montt</t>
-        </is>
-      </c>
-      <c r="H432" s="14" t="inlineStr">
-        <is>
-          <t>977745392/921776772</t>
-        </is>
-      </c>
-      <c r="I432" s="14" t="inlineStr">
-        <is>
-          <t>cliente ingresado automaticamente</t>
-        </is>
-      </c>
-      <c r="J432" s="14" t="n">
-        <v>10062</v>
-      </c>
-      <c r="K432" s="14" t="inlineStr">
-        <is>
-          <t>REALIZADO</t>
-        </is>
-      </c>
-      <c r="L432" s="14" t="inlineStr">
-        <is>
-          <t>ca3l10 ba10 mensaje extra</t>
-        </is>
-      </c>
-      <c r="Z432" s="14" t="n">
-        <v>10</v>
-      </c>
-      <c r="AF432" s="14" t="n">
-        <v>10</v>
-      </c>
-      <c r="AI432" s="14" t="inlineStr">
-        <is>
-          <t>Ruta: Osorno-LaUnion-RioBueno-Valdivia</t>
-        </is>
-      </c>
-    </row>
+    <row r="431" ht="15" customHeight="1" s="15"/>
+    <row r="432" ht="15" customHeight="1" s="15"/>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Nueva ruta publica y ajustes en funcionamiento js de rutabd
</commit_message>
<xml_diff>
--- a/bd/mediclean_bd.xlsx
+++ b/bd/mediclean_bd.xlsx
@@ -615,7 +615,7 @@
       </c>
       <c r="C2" s="17" t="inlineStr">
         <is>
-          <t>Aqa1XLWSxZtU1jzgz9xIzrrYT5KxIkvADqR9yiSP4CQ</t>
+          <t>hfOaXUiL3TITsSehJ-Q4vkh0VhE0Gg0YsjhmLEBjFFA</t>
         </is>
       </c>
     </row>
@@ -11425,7 +11425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AN431"/>
+  <dimension ref="A1:AN430"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.59375" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8.699999999999999" customWidth="1" style="14" min="1" max="1"/>

</xml_diff>